<commit_message>
docs: set the paper-forward observation window
</commit_message>
<xml_diff>
--- a/picks.xlsx
+++ b/picks.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Picks" sheetId="1" r:id="Rdc210d98d1c74c8a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Track Record" sheetId="2" r:id="R1d9541f815ad464e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How To Read This" sheetId="3" r:id="R6dab8729227540b4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Research Status" sheetId="4" r:id="R1506efc22b4e48dc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Picks" sheetId="1" r:id="Rf1c92a74b0a74060"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Track Record" sheetId="2" r:id="R4bff5232c2b843b3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How To Read This" sheetId="3" r:id="R8cc0b2fa22a4455d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Research Status" sheetId="4" r:id="Rfee08e634413478d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4691,7 +4691,9 @@
       </x:c>
     </x:row>
     <x:row r="17">
-      <x:c r="A17" s="89" t="str"/>
+      <x:c r="A17" s="89" t="str">
+        <x:v>Track a frozen candidate for at least six months; twelve months is the default, and a longer written gate wins.</x:v>
+      </x:c>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="93" t="str">

</xml_diff>